<commit_message>
Improve company ranking and web crawler
</commit_message>
<xml_diff>
--- a/output/dataset/market_gap_dataset.xlsx
+++ b/output/dataset/market_gap_dataset.xlsx
@@ -1924,99 +1924,87 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>AI Solutions</t>
+          <t>AI Consulting</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Insight accelerates transformation by unlocking the power of people and technology. We drive speed, scale, resilience, and innovation to help clients achieve their ambitious goals.</t>
+          <t>Insight accelerates transformation by unlocking the power of people and technology. We serve the public and private sectors, providing deep industry experience and technical skills to guide your organization's IT transformation goals. Our AI consulting services include Insight Prism, helping identify high-value use cases and define a clear path forward.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>Build your AI roadmap</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Cloud Platforms, Databases, DevOps Tools, AI Frameworks, LLMs</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>No Computer Vision Solutions, Limited AI Adoption</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Computer Vision Platform, AI for Computer Vision</t>
-        </is>
-      </c>
+          <t>No. 427 Fortune 500</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Python, AI, Machine Learning, Computer Vision</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>pandas, matplotlib, numpy, object detection, image detection</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Python, React Native, PyTorch, Computer Vision, Natural Language Processing (NLP), Mobile Application Development</t>
+          <t>Strong Python and AI skills</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Add Computer Vision skills to the profile</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>Computer Vision Solutions</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+          <t>Expand skill set with additional technologies like pandas, matplotlib, numpy, object detection, image detection</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>aima khan</t>
+          <t>Aima Khan</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>CV Engineer</t>
         </is>
       </c>
       <c r="U19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y19" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="W19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="X19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Z19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Add content cleaning, duplicate detection, evidence records and unit tests
</commit_message>
<xml_diff>
--- a/output/dataset/market_gap_dataset.xlsx
+++ b/output/dataset/market_gap_dataset.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Gap Dataset" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Market Gap Dataset'!$A$1:$Z$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Market Gap Dataset'!$A$1:$Z$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z35"/>
+  <dimension ref="A1:Z37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2497,27 +2497,31 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Python, Machine Learning, AI Algorithms, Deep Learning, Computer Vision</t>
+        </is>
+      </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Java, Docker, Kubernetes</t>
+          <t>project management, tensorflow, pytorch</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Python, React Native, PyTorch, Computer Vision, Natural Language Processing (NLP), Mobile Application Development</t>
+          <t>Strong in Python and related technologies</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Java, Docker, Kubernetes</t>
+          <t>Expand skills in project management, TensorFlow, PyTorch</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -2532,12 +2536,12 @@
       <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>aima khan</t>
+          <t>Aima Khan</t>
         </is>
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="U25" s="2" t="n">
@@ -2550,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y25" s="2" t="n">
         <v>3</v>
@@ -3344,155 +3348,359 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Vedia Cloud Analytics</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>https://vedia.ca/machinelearning-solutions/</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>AI Solutions</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Unlock the potential of machine learning with our tailored solutions, including predictive modeling, classification, clustering, and anomaly detection. Vedia’s machine learning services encompass the entire lifecycle of designing, building, and deploying customized solutions tailored to your business needs.</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>AI software development, AI consulting services, Computer vision consulting, Machine learning consulting, NLP consulting, AI readiness assessment</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>AWS, Azure, Google Cloud, Salesforce, SharePoint</t>
-        </is>
-      </c>
+          <t>Predictive Modeling, Classification, Clustering, Anomaly Detection, Regression Analysis</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Manual workflows, Limited automation, Poor personalization, No chatbot, No AI-driven insights</t>
+          <t>No AI-driven insights, Poor personalization</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Docker, AWS</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Python, Machine Learning, Full Stack Web Development, TensorFlow, PyTorch</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Docker, AWS</t>
+        </is>
+      </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>AI Chatbot Development, Predictive Analytics, Automation Solutions</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
+          <t>Predictive Modeling, Classification, Clustering, Anomaly Detection, Regression Analysis</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr"/>
-      <c r="T34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>Aima Khan</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
       <c r="U34" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="X34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z34" s="2" t="n">
         <v>5</v>
-      </c>
-      <c r="W34" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="X34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z34" s="2" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>viso.ai</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>https://viso.ai/computer-vision/most-popular-computer-vision-companies-and-startups/</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Computer Vision Software Companies</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>viso.ai is a computer vision company from Switzerland that provides the world's only end-to-end computer vision platform, Viso Suite. Using this solution, teams can build, deploy, and scale all their computer vision applications on one unified infrastructure.</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Computer Vision Infrastructure</t>
+          <t>AI software development, AI consulting services, Computer vision consulting, Machine learning consulting, NLP consulting, AI readiness assessment</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Python, Java, FastAPI, TensorFlow, PyTorch, AWS, Azure, Docker, Kubernetes, AI Frameworks, LLMs</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr"/>
+          <t>AWS, Azure, Google Cloud, Salesforce, SharePoint</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Manual workflows, Limited automation, Poor personalization, No chatbot, No AI-driven insights</t>
+        </is>
+      </c>
       <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Python, React Native, PyTorch, Computer Vision, Natural Language Processing (NLP)</t>
-        </is>
-      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>Strong Python skills, Experience in React Native and PyTorch</t>
-        </is>
-      </c>
+      <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
+          <t>AI Chatbot Development, Predictive Analytics, Automation Solutions</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="inlineStr"/>
+      <c r="T35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="V35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="W35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="X35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>viso.ai</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>https://viso.ai/computer-vision/most-popular-computer-vision-companies-and-startups/</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Computer Vision Software Companies</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>viso.ai is a computer vision company from Switzerland that provides the world's only end-to-end computer vision platform, Viso Suite. Using this solution, teams can build, deploy, and scale all their computer vision applications on one unified infrastructure.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Computer Vision Infrastructure</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Python, Java, FastAPI, TensorFlow, PyTorch, AWS, Azure, Docker, Kubernetes, AI Frameworks, LLMs</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Python, React Native, PyTorch, Computer Vision, Natural Language Processing (NLP)</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Strong Python skills, Experience in React Native and PyTorch</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
           <t>AI Chatbot Development, Computer Vision Solutions</t>
         </is>
       </c>
-      <c r="P35" s="2" t="inlineStr"/>
-      <c r="Q35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="2" t="inlineStr"/>
-      <c r="S35" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr">
         <is>
           <t>aima khan</t>
         </is>
       </c>
-      <c r="T35" s="2" t="inlineStr">
+      <c r="T36" s="2" t="inlineStr">
         <is>
           <t>Frontend Developer</t>
         </is>
       </c>
-      <c r="U35" s="2" t="n">
+      <c r="U36" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V35" s="2" t="n">
+      <c r="V36" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="W35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X35" s="2" t="n">
+      <c r="W36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="Y35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z35" s="2" t="n">
+      <c r="Y36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Width.ai</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.width.ai/</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Machine Learning Consulting</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Width.ai is an AI &amp; Machine Learning consulting company focused on generative ai implementations. We help companies build ai projects through development and strategy.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Computer Vision, Ai Chatbots, Object Detection, Prompt Engineering, NLP Services</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Python, Java, FastAPI, TensorFlow, PyTorch, AWS, Azure, Docker, Kubernetes</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>No AI-driven insights, Limited automation, No chatbot</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>AI Chatbot, Recommendation Systems, Predictive Analytics</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Python, Machine Learning, AI Algorithms, Deep Learning, Computer Vision</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Strong Python and Machine Learning skills, Broad AI skill set including deep learning, computer vision, and project management</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation Systems, Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>Aima Khan</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="V37" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="W37" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="X37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="2" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z35"/>
+  <autoFilter ref="A1:Z37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>